<commit_message>
dia 19 y 17
</commit_message>
<xml_diff>
--- a/horas.xlsx
+++ b/horas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wenji\Desktop\DSA\EA_ViveBook_TeamManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E9A50A3-2FAE-4B72-AE4C-C1556E328A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90C1B6C1-8997-4B94-9F5F-6DB9D641A803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="119">
   <si>
     <t>UPC - EETAC - EA-M QP2526 Grup 3: Còmput de les hores de treball del projecte ViveBook</t>
   </si>
@@ -390,6 +390,15 @@
   </si>
   <si>
     <t>Home Page fixed, Profile Avatar implemented</t>
+  </si>
+  <si>
+    <t>Image upload fixed and Adding Book event matomo</t>
+  </si>
+  <si>
+    <t>Fixes openlibrary api</t>
+  </si>
+  <si>
+    <t>Fixes Create Libro Modal</t>
   </si>
 </sst>
 </file>
@@ -2591,19 +2600,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>116.5</c:v>
+                  <c:v>118.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>40.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>43</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>77.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>118</c:v>
+                  <c:v>119</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4645,19 +4654,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>32</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>21.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>25</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9233,12 +9242,12 @@
       </c>
       <c r="H6" s="63">
         <f>SUM(WENJIE!F5:F138)</f>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I6" s="30"/>
       <c r="J6" s="31">
         <f>SUM(D6:H6)</f>
-        <v>116.5</v>
+        <v>118.5</v>
       </c>
       <c r="K6" s="20"/>
     </row>
@@ -9321,12 +9330,12 @@
       </c>
       <c r="H10" s="69">
         <f>SUM(WENJIE!L5:L138)</f>
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I10" s="41"/>
       <c r="J10" s="42">
         <f>SUM(D10:H10)</f>
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="K10" s="20"/>
     </row>
@@ -9409,12 +9418,12 @@
       </c>
       <c r="H14" s="75">
         <f>SUM(WENJIE!R5:R138)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I14" s="49"/>
       <c r="J14" s="50">
         <f>SUM(D14:H14)</f>
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K14" s="20"/>
     </row>
@@ -9452,12 +9461,12 @@
       </c>
       <c r="H16" s="18">
         <f>SUM(H6:H14)</f>
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I16" s="23"/>
       <c r="J16" s="18">
         <f>SUM(D16:H16)</f>
-        <v>395.5</v>
+        <v>404.5</v>
       </c>
     </row>
     <row r="22" spans="5:11" x14ac:dyDescent="0.25">
@@ -27242,7 +27251,7 @@
     <col min="10" max="10" width="35.5703125" style="7" customWidth="1"/>
     <col min="11" max="11" width="2.5703125" style="1" customWidth="1"/>
     <col min="12" max="12" width="5.140625" style="2" customWidth="1"/>
-    <col min="13" max="13" width="35.5703125" style="8" customWidth="1"/>
+    <col min="13" max="13" width="54" style="8" customWidth="1"/>
     <col min="14" max="14" width="2.5703125" style="1" customWidth="1"/>
     <col min="15" max="15" width="5.140625" style="2" customWidth="1"/>
     <col min="16" max="16" width="35.5703125" style="9" customWidth="1"/>
@@ -31473,9 +31482,11 @@
       <c r="J133" s="57"/>
       <c r="K133" s="90"/>
       <c r="L133" s="78">
-        <v>0</v>
-      </c>
-      <c r="M133" s="58"/>
+        <v>4</v>
+      </c>
+      <c r="M133" s="58" t="s">
+        <v>116</v>
+      </c>
       <c r="N133" s="90"/>
       <c r="O133" s="79">
         <v>0</v>
@@ -31483,9 +31494,11 @@
       <c r="P133" s="59"/>
       <c r="Q133" s="90"/>
       <c r="R133" s="80">
-        <v>0</v>
-      </c>
-      <c r="S133" s="60"/>
+        <v>1</v>
+      </c>
+      <c r="S133" s="60" t="s">
+        <v>112</v>
+      </c>
       <c r="U133" s="14"/>
       <c r="V133" s="14"/>
     </row>
@@ -31527,9 +31540,11 @@
         <v>19</v>
       </c>
       <c r="F135" s="76">
-        <v>0</v>
-      </c>
-      <c r="G135" s="4"/>
+        <v>2</v>
+      </c>
+      <c r="G135" s="4" t="s">
+        <v>117</v>
+      </c>
       <c r="H135" s="90"/>
       <c r="I135" s="77">
         <v>0</v>
@@ -31537,9 +31552,11 @@
       <c r="J135" s="57"/>
       <c r="K135" s="90"/>
       <c r="L135" s="78">
-        <v>0</v>
-      </c>
-      <c r="M135" s="58"/>
+        <v>2</v>
+      </c>
+      <c r="M135" s="58" t="s">
+        <v>118</v>
+      </c>
       <c r="N135" s="90"/>
       <c r="O135" s="79">
         <v>0</v>

</xml_diff>